<commit_message>
observation and analysis form ready
</commit_message>
<xml_diff>
--- a/templates/analysis-form.xlsx
+++ b/templates/analysis-form.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eklem/github_modules/usability-testing-kit/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FAE3B1E-408A-9B45-8258-526161175895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F4F5C34-EEC9-1546-AE28-CE6C247DABB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-18180" yWindow="-28300" windowWidth="68800" windowHeight="28300" xr2:uid="{F49927BD-70D1-124E-B412-3DEFD0188356}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{F49927BD-70D1-124E-B412-3DEFD0188356}"/>
   </bookViews>
   <sheets>
     <sheet name="User #" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Context/
 Place in application</t>
@@ -64,6 +64,23 @@
   </si>
   <si>
     <t>Usability test analysis - [name of test] - Number of users: [#]</t>
+  </si>
+  <si>
+    <t>Possible causes</t>
+  </si>
+  <si>
+    <t>Possible solutions</t>
+  </si>
+  <si>
+    <t>Effort to solve
+(1-3)</t>
+  </si>
+  <si>
+    <t>Priority
+(1-n)</t>
+  </si>
+  <si>
+    <t>Added to backlog (x)</t>
   </si>
 </sst>
 </file>
@@ -155,14 +172,19 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -186,9 +208,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -226,7 +248,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -332,7 +354,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -474,7 +496,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -482,7 +504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F10F915B-4AB4-3E4B-9783-CF8B22243770}">
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="50.33203125" customWidth="1"/>
@@ -490,112 +512,213 @@
     <col min="4" max="4" width="11.6640625" customWidth="1"/>
     <col min="5" max="5" width="13.33203125" customWidth="1"/>
     <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="74.83203125" customWidth="1"/>
+    <col min="9" max="9" width="74.33203125" customWidth="1"/>
+    <col min="10" max="10" width="18.5" customWidth="1"/>
+    <col min="12" max="12" width="14.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="24" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
-    </row>
-    <row r="2" spans="1:15" ht="50" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+    </row>
+    <row r="2" spans="1:12" ht="75" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-    </row>
-    <row r="3" spans="1:15" ht="24" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+      <c r="H2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-    </row>
-    <row r="4" spans="1:15" ht="24" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+    </row>
+    <row r="4" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-    </row>
-    <row r="5" spans="1:15" ht="24" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+    </row>
+    <row r="5" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A5" s="4">
         <v>3</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-    </row>
-    <row r="6" spans="1:15" ht="24" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+    </row>
+    <row r="6" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A6" s="4">
         <v>4</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-    </row>
-    <row r="7" spans="1:15" ht="24" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+    </row>
+    <row r="7" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A7" s="4">
         <v>5</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-    </row>
-    <row r="8" spans="1:15" ht="24" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+    </row>
+    <row r="8" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A8" s="4">
         <v>6</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-    </row>
-    <row r="9" spans="1:15" ht="24" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+    </row>
+    <row r="9" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A9" s="4">
         <v>7</v>
       </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-    </row>
-    <row r="10" spans="1:15" ht="24" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+    </row>
+    <row r="10" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A10" s="4">
         <v>8</v>
       </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-    </row>
-    <row r="11" spans="1:15" ht="24" x14ac:dyDescent="0.3">
-      <c r="A11" s="1">
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+    </row>
+    <row r="11" spans="1:12" ht="24" x14ac:dyDescent="0.3">
+      <c r="A11" s="4">
         <v>9</v>
       </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>